<commit_message>
Refactor analytics seed tests to include new models and improve count logic; add comprehensive documentation structure for onboarding, API, architecture, and security; update user onboarding form creation process and remove outdated onboarding documentation.
</commit_message>
<xml_diff>
--- a/docs/onboarding/bountyflow-onboarding.xlsx
+++ b/docs/onboarding/bountyflow-onboarding.xlsx
@@ -13,10 +13,10 @@
     <sheet name="Form responses" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$B$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Participants'!$A$1:$I$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'In-product feedback'!$A$1:$K$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Form responses'!$A$3:$H$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$B$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Participants'!$A$1:$I$66</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'In-product feedback'!$A$1:$K$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Form responses'!$A$3:$K$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -479,7 +479,7 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>9</v>
+        <v>65</v>
       </c>
     </row>
     <row r="3">
@@ -499,7 +499,7 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>2</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5">
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>5</v>
+        <v>49</v>
       </c>
     </row>
     <row r="6">
@@ -519,7 +519,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>1</v>
+        <v>50</v>
       </c>
     </row>
     <row r="7">
@@ -529,7 +529,7 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8">
@@ -539,7 +539,7 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>1</v>
+        <v>26</v>
       </c>
     </row>
     <row r="9">
@@ -559,21 +559,51 @@
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>46295.00019014891</v>
+        <v>46295.02134853722</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
+          <t>Feedback — Bug</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Feedback — Idea</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Feedback — Other</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
           <t>Feedback — Praise</t>
         </is>
       </c>
-      <c r="B11" s="2" t="n">
-        <v>1</v>
+      <c r="B14" s="2" t="n">
+        <v>11</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B11"/>
+  <autoFilter ref="A1:B14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -584,7 +614,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -974,8 +1004,2100 @@
         <v>46294.66400265676</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Helio Collective</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>helio-collective</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>helio.collective@bountyflow.test</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr"/>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr"/>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I11" s="5" t="n">
+        <v>46295.01508319439</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Aurora Ledger</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>aurora-ledger</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>aurora.ledger@bountyflow.test</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr"/>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr"/>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="n">
+        <v>46295.0150839757</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Fatima El Amrani</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>fatima-el-amrani</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>fatima.el.amrani@bountyflow.test</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr"/>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr"/>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I13" s="5" t="n">
+        <v>46295.01508405559</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Lucas Ferreira</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>lucas-ferreira</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>lucas.ferreira@bountyflow.test</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr"/>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr"/>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="n">
+        <v>46295.01508414634</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Anneke Visser</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>anneke-visser</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>anneke.visser@bountyflow.test</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr"/>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr"/>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I15" s="5" t="n">
+        <v>46295.01508424328</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Hiroshi Endō</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>hiroshi-endo</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>hiroshi.endo@bountyflow.test</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr"/>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr"/>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="n">
+        <v>46295.01508432844</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Dilnoza Usmanova</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>dilnoza-usmanova</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>dilnoza.usmanova@bountyflow.test</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr"/>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr"/>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I17" s="5" t="n">
+        <v>46295.01508442551</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Noor Rahman</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>noor-rahman</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>noor.rahman@bountyflow.test</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr"/>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr"/>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I18" s="5" t="n">
+        <v>46295.01508450114</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Théo Lambert</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>theo-lambert</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>theo.lambert@bountyflow.test</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr"/>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr"/>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I19" s="5" t="n">
+        <v>46295.01508462529</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Zanele Mthembu</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>zanele-mthembu</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>zanele.mthembu@bountyflow.test</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr"/>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="inlineStr"/>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I20" s="5" t="n">
+        <v>46295.01508469928</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Arun Ramaswamy</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>arun-ramaswamy</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>arun.ramaswamy@bountyflow.test</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr"/>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr"/>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I21" s="5" t="n">
+        <v>46295.01508480838</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Inès Moreau</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>ines-moreau</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>ines.moreau@bountyflow.test</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr"/>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H22" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I22" s="5" t="n">
+        <v>46295.01508488268</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Piotr Kaczmarek</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>piotr-kaczmarek</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>piotr.kaczmarek@bountyflow.test</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr"/>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr"/>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I23" s="5" t="n">
+        <v>46295.01508495361</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Kwame Asante</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>kwame-asante</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>kwame.asante@bountyflow.test</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr"/>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I24" s="5" t="n">
+        <v>46295.01508502369</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Siti Rahayu</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>siti-rahayu</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>siti.rahayu@bountyflow.test</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr"/>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I25" s="5" t="n">
+        <v>46295.01508510919</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Matías Ovalle</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>matias-ovalle</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>matias.ovalle@bountyflow.test</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr"/>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H26" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I26" s="5" t="n">
+        <v>46295.01508522841</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Grace Wanjiru</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>grace-wanjiru</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>grace.wanjiru@bountyflow.test</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr"/>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I27" s="5" t="n">
+        <v>46295.01508532763</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Yusuf Bello</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>yusuf-bello</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>yusuf.bello@bountyflow.test</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr"/>
+      <c r="F28" s="4" t="inlineStr"/>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H28" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I28" s="5" t="n">
+        <v>46295.01508541921</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Elena Petrova</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>elena-petrova</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>elena.petrova@bountyflow.test</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr"/>
+      <c r="F29" s="4" t="inlineStr"/>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H29" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I29" s="5" t="n">
+        <v>46295.01508550565</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Mateo Silva</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>mateo-silva</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>mateo.silva@bountyflow.test</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr"/>
+      <c r="F30" s="4" t="inlineStr"/>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H30" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I30" s="5" t="n">
+        <v>46295.01508558371</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Aiko Matsumoto</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>aiko-matsumoto</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>aiko.matsumoto@bountyflow.test</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr"/>
+      <c r="F31" s="4" t="inlineStr"/>
+      <c r="G31" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H31" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I31" s="5" t="n">
+        <v>46295.01508565892</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Daniel Okonkwo</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>daniel-okonkwo</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>daniel.okonkwo@bountyflow.test</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="inlineStr"/>
+      <c r="F32" s="4" t="inlineStr"/>
+      <c r="G32" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H32" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I32" s="5" t="n">
+        <v>46295.01508573463</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Sana Qureshi</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>sana-qureshi</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>sana.qureshi@bountyflow.test</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr"/>
+      <c r="F33" s="4" t="inlineStr"/>
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H33" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I33" s="5" t="n">
+        <v>46295.01508580272</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Linh Nguyễn</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>linh-nguyen</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>linh.nguyen@bountyflow.test</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="inlineStr"/>
+      <c r="F34" s="4" t="inlineStr"/>
+      <c r="G34" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H34" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I34" s="5" t="n">
+        <v>46295.01508587464</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Oscar Lindqvist</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>oscar-lindqvist</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>oscar.lindqvist@bountyflow.test</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr"/>
+      <c r="F35" s="4" t="inlineStr"/>
+      <c r="G35" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H35" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I35" s="5" t="n">
+        <v>46295.01508596077</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Amara Diallo</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>amara-diallo</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>amara.diallo@bountyflow.test</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="inlineStr"/>
+      <c r="F36" s="4" t="inlineStr"/>
+      <c r="G36" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H36" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I36" s="5" t="n">
+        <v>46295.01508604862</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Ravi Deshmukh</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>ravi-deshmukh</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>ravi.deshmukh@bountyflow.test</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr"/>
+      <c r="F37" s="4" t="inlineStr"/>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H37" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I37" s="5" t="n">
+        <v>46295.01508618319</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Nina Schneider</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>nina-schneider</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>nina.schneider@bountyflow.test</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr"/>
+      <c r="F38" s="4" t="inlineStr"/>
+      <c r="G38" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H38" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I38" s="5" t="n">
+        <v>46295.01508626442</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Tobias Berg</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>tobias-berg</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>tobias.berg@bountyflow.test</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr"/>
+      <c r="F39" s="4" t="inlineStr"/>
+      <c r="G39" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H39" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I39" s="5" t="n">
+        <v>46295.01508633742</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>Carmen Ortiz</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>carmen-ortiz</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>carmen.ortiz@bountyflow.test</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr"/>
+      <c r="F40" s="4" t="inlineStr"/>
+      <c r="G40" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H40" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I40" s="5" t="n">
+        <v>46295.0150864083</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>Wei Zhang</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>wei-zhang</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>wei.zhang@bountyflow.test</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr"/>
+      <c r="F41" s="4" t="inlineStr"/>
+      <c r="G41" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H41" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I41" s="5" t="n">
+        <v>46295.01508648063</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Gabriel Mensah</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>gabriel-mensah</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>gabriel.mensah@bountyflow.test</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="inlineStr"/>
+      <c r="F42" s="4" t="inlineStr"/>
+      <c r="G42" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H42" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I42" s="5" t="n">
+        <v>46295.01508655877</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>Isabela Rocha</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>isabela-rocha</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>isabela.rocha@bountyflow.test</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr"/>
+      <c r="F43" s="4" t="inlineStr"/>
+      <c r="G43" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H43" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I43" s="5" t="n">
+        <v>46295.01508663064</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Omar Haddad</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>omar-haddad</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>omar.haddad@bountyflow.test</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr"/>
+      <c r="F44" s="4" t="inlineStr"/>
+      <c r="G44" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H44" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I44" s="5" t="n">
+        <v>46295.01508672137</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>Freya Nilsen</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>freya-nilsen</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>freya.nilsen@bountyflow.test</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="inlineStr"/>
+      <c r="F45" s="4" t="inlineStr"/>
+      <c r="G45" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H45" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I45" s="5" t="n">
+        <v>46295.01508680662</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>Karan Mehta</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>karan-mehta</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>karan.mehta@bountyflow.test</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E46" s="4" t="inlineStr"/>
+      <c r="F46" s="4" t="inlineStr"/>
+      <c r="G46" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H46" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I46" s="5" t="n">
+        <v>46295.01508689395</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>Hana Suzuki</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>hana-suzuki</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>hana.suzuki@bountyflow.test</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="inlineStr"/>
+      <c r="F47" s="4" t="inlineStr"/>
+      <c r="G47" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H47" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I47" s="5" t="n">
+        <v>46295.01508697702</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>Emeka Nwosu</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>emeka-nwosu</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>emeka.nwosu@bountyflow.test</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E48" s="4" t="inlineStr"/>
+      <c r="F48" s="4" t="inlineStr"/>
+      <c r="G48" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H48" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I48" s="5" t="n">
+        <v>46295.01508706501</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>Lior Ben-Ami</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>lior-ben-ami</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
+          <t>lior.ben.ami@bountyflow.test</t>
+        </is>
+      </c>
+      <c r="D49" s="4" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E49" s="4" t="inlineStr"/>
+      <c r="F49" s="4" t="inlineStr"/>
+      <c r="G49" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H49" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I49" s="5" t="n">
+        <v>46295.01508713725</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>Marta Kowalska</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>marta-kowalska</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t>marta.kowalska@bountyflow.test</t>
+        </is>
+      </c>
+      <c r="D50" s="4" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E50" s="4" t="inlineStr"/>
+      <c r="F50" s="4" t="inlineStr"/>
+      <c r="G50" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H50" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I50" s="5" t="n">
+        <v>46295.01508720776</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>Ahmed Farouk</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>ahmed-farouk</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>ahmed.farouk@bountyflow.test</t>
+        </is>
+      </c>
+      <c r="D51" s="4" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E51" s="4" t="inlineStr"/>
+      <c r="F51" s="4" t="inlineStr"/>
+      <c r="G51" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H51" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I51" s="5" t="n">
+        <v>46295.01508728264</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>Sofia Marchetti</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>sofia-marchetti</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
+          <t>sofia.marchetti@bountyflow.test</t>
+        </is>
+      </c>
+      <c r="D52" s="4" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E52" s="4" t="inlineStr"/>
+      <c r="F52" s="4" t="inlineStr"/>
+      <c r="G52" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H52" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I52" s="5" t="n">
+        <v>46295.01508735148</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>Tariq Benali</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>tariq-benali</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="inlineStr">
+        <is>
+          <t>tariq.benali@bountyflow.test</t>
+        </is>
+      </c>
+      <c r="D53" s="4" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E53" s="4" t="inlineStr"/>
+      <c r="F53" s="4" t="inlineStr"/>
+      <c r="G53" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H53" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I53" s="5" t="n">
+        <v>46295.01508741773</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>Mei-Lin Koh</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>mei-lin-koh</t>
+        </is>
+      </c>
+      <c r="C54" s="4" t="inlineStr">
+        <is>
+          <t>mei.lin.koh@bountyflow.test</t>
+        </is>
+      </c>
+      <c r="D54" s="4" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E54" s="4" t="inlineStr"/>
+      <c r="F54" s="4" t="inlineStr"/>
+      <c r="G54" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H54" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I54" s="5" t="n">
+        <v>46295.01508748843</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>Pablo Navarro</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>pablo-navarro</t>
+        </is>
+      </c>
+      <c r="C55" s="4" t="inlineStr">
+        <is>
+          <t>pablo.navarro@bountyflow.test</t>
+        </is>
+      </c>
+      <c r="D55" s="4" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E55" s="4" t="inlineStr"/>
+      <c r="F55" s="4" t="inlineStr"/>
+      <c r="G55" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H55" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I55" s="5" t="n">
+        <v>46295.01508756414</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>Zara Iqbal</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>zara-iqbal</t>
+        </is>
+      </c>
+      <c r="C56" s="4" t="inlineStr">
+        <is>
+          <t>zara.iqbal@bountyflow.test</t>
+        </is>
+      </c>
+      <c r="D56" s="4" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E56" s="4" t="inlineStr"/>
+      <c r="F56" s="4" t="inlineStr"/>
+      <c r="G56" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H56" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I56" s="5" t="n">
+        <v>46295.01508763921</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>Ana Melo</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>ana-melo</t>
+        </is>
+      </c>
+      <c r="C57" s="4" t="inlineStr">
+        <is>
+          <t>ana.melo@bountyflow.test</t>
+        </is>
+      </c>
+      <c r="D57" s="4" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E57" s="4" t="inlineStr"/>
+      <c r="F57" s="4" t="inlineStr"/>
+      <c r="G57" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H57" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I57" s="5" t="n">
+        <v>46295.01508770735</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>Jonas Weber</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>jonas-weber</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="inlineStr">
+        <is>
+          <t>jonas.weber@bountyflow.test</t>
+        </is>
+      </c>
+      <c r="D58" s="4" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E58" s="4" t="inlineStr"/>
+      <c r="F58" s="4" t="inlineStr"/>
+      <c r="G58" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H58" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I58" s="5" t="n">
+        <v>46295.01508778213</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>Leila Haddadi</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>leila-haddadi</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="inlineStr">
+        <is>
+          <t>leila.haddadi@bountyflow.test</t>
+        </is>
+      </c>
+      <c r="D59" s="4" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E59" s="4" t="inlineStr"/>
+      <c r="F59" s="4" t="inlineStr"/>
+      <c r="G59" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H59" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I59" s="5" t="n">
+        <v>46295.01508785816</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>Daniela Vargas</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>daniela-vargas</t>
+        </is>
+      </c>
+      <c r="C60" s="4" t="inlineStr">
+        <is>
+          <t>daniela.vargas@bountyflow.test</t>
+        </is>
+      </c>
+      <c r="D60" s="4" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E60" s="4" t="inlineStr"/>
+      <c r="F60" s="4" t="inlineStr"/>
+      <c r="G60" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H60" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I60" s="5" t="n">
+        <v>46295.01508797333</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>Samuel Adeniyi</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>samuel-adeniyi</t>
+        </is>
+      </c>
+      <c r="C61" s="4" t="inlineStr">
+        <is>
+          <t>samuel.adeniyi@bountyflow.test</t>
+        </is>
+      </c>
+      <c r="D61" s="4" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E61" s="4" t="inlineStr"/>
+      <c r="F61" s="4" t="inlineStr"/>
+      <c r="G61" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H61" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I61" s="5" t="n">
+        <v>46295.01508806109</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>Natalia Sokolova</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>natalia-sokolova</t>
+        </is>
+      </c>
+      <c r="C62" s="4" t="inlineStr">
+        <is>
+          <t>natalia.sokolova@bountyflow.test</t>
+        </is>
+      </c>
+      <c r="D62" s="4" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E62" s="4" t="inlineStr"/>
+      <c r="F62" s="4" t="inlineStr"/>
+      <c r="G62" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H62" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I62" s="5" t="n">
+        <v>46295.01508813279</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>Arjun Pillai</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>arjun-pillai</t>
+        </is>
+      </c>
+      <c r="C63" s="4" t="inlineStr">
+        <is>
+          <t>arjun.pillai@bountyflow.test</t>
+        </is>
+      </c>
+      <c r="D63" s="4" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E63" s="4" t="inlineStr"/>
+      <c r="F63" s="4" t="inlineStr"/>
+      <c r="G63" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H63" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I63" s="5" t="n">
+        <v>46295.01508820501</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>Maya Goldberg</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>maya-goldberg</t>
+        </is>
+      </c>
+      <c r="C64" s="4" t="inlineStr">
+        <is>
+          <t>maya.goldberg@bountyflow.test</t>
+        </is>
+      </c>
+      <c r="D64" s="4" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E64" s="4" t="inlineStr"/>
+      <c r="F64" s="4" t="inlineStr"/>
+      <c r="G64" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H64" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I64" s="5" t="n">
+        <v>46295.01508828194</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>Felipe Cardozo</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>felipe-cardozo</t>
+        </is>
+      </c>
+      <c r="C65" s="4" t="inlineStr">
+        <is>
+          <t>felipe.cardozo@bountyflow.test</t>
+        </is>
+      </c>
+      <c r="D65" s="4" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E65" s="4" t="inlineStr"/>
+      <c r="F65" s="4" t="inlineStr"/>
+      <c r="G65" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H65" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I65" s="5" t="n">
+        <v>46295.01508835087</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>Aminata Traoré</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>aminata-traore</t>
+        </is>
+      </c>
+      <c r="C66" s="4" t="inlineStr">
+        <is>
+          <t>aminata.traore@bountyflow.test</t>
+        </is>
+      </c>
+      <c r="D66" s="4" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E66" s="4" t="inlineStr"/>
+      <c r="F66" s="4" t="inlineStr"/>
+      <c r="G66" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H66" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I66" s="5" t="n">
+        <v>46295.01508842788</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I10"/>
+  <autoFilter ref="A1:I66"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -986,7 +3108,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1098,8 +3220,2191 @@
       <c r="J2" s="4" t="inlineStr"/>
       <c r="K2" s="4" t="inlineStr"/>
     </row>
+    <row r="3">
+      <c r="A3" s="3" t="n">
+        <v>46294.8901581021</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>If I filter the marketplace by category and then open a bounty and press back, every filter is gone and I am at the top of the list again. I lose my place every single time.</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>Mateo Silva</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr"/>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>/bounties</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>1920 x 947</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="n"/>
+      <c r="J3" s="4" t="inlineStr"/>
+      <c r="K3" s="4" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="n">
+        <v>46294.80682476876</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Let me save a search from the marketplace in one click instead of going to the saved page and rebuilding the filters by hand. The filters are already on screen.</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Isabela Rocha</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr"/>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>/bounties</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>1920 x 947</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="n"/>
+      <c r="J4" s="4" t="inlineStr"/>
+      <c r="K4" s="4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="n">
+        <v>46294.72349143543</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>A notification about a reply on my question links to the bounty but not to the question itself, so on a long thread I have to hunt for what changed.</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Gabriel Mensah</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr"/>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>/app/notifications</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>1440 x 768</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="n"/>
+      <c r="J5" s="4" t="inlineStr"/>
+      <c r="K5" s="4" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="n">
+        <v>46294.6859429545</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Praise</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>The questions section on a bounty is the best thing here. I got a clear answer about scope in three hours and it stopped me writing an application for the wrong job.</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Yusuf Bello</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr"/>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>/bounties/security-review-of-a-soroban-token-vesting-contract-c15755</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>1512 x 857</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="n"/>
+      <c r="J6" s="4" t="inlineStr"/>
+      <c r="K6" s="4" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="n">
+        <v>46294.6401581021</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Handled</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Sorting by reward puts a 90 XLM bounty above a 1200 one. Looks like it is sorting the amount as text rather than as a number.</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Arjun Pillai</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr"/>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>/bounties</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>2560 x 1329</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="n">
+        <v>46294.80682476876</v>
+      </c>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>Morgan Reyes</t>
+        </is>
+      </c>
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>Confirmed — the sort was comparing the formatted string. Fixed in this week's release and I replied to Arjun directly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="n">
+        <v>46294.5609429545</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>The cover letter box does not tell you the character limit until you exceed it, and then it just refuses to submit without saying by how much.</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Tariq Benali</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr"/>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>/bounties/build-a-webhook-delivery-service-with-exponential-backoff-817fd0</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>412 x 823</t>
+        </is>
+      </c>
+      <c r="I8" s="4" t="n"/>
+      <c r="J8" s="4" t="inlineStr"/>
+      <c r="K8" s="4" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="n">
+        <v>46294.5151581021</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Keyboard shortcuts for the marketplace — j and k to move between results, enter to open. I browse this list a lot.</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Elena Petrova</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr"/>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>/bounties</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>2560 x 1329</t>
+        </is>
+      </c>
+      <c r="I9" s="4" t="n"/>
+      <c r="J9" s="4" t="inlineStr"/>
+      <c r="K9" s="4" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="n">
+        <v>46294.47349143543</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>The difficulty labels mean different things to different requesters. A one-line definition on hover would help people apply to the right things.</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Anonymous</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>p.okoye.writes@example.test</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>/how-it-works</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>1366 x 625</t>
+        </is>
+      </c>
+      <c r="I10" s="4" t="n"/>
+      <c r="J10" s="4" t="inlineStr"/>
+      <c r="K10" s="4" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="n">
+        <v>46294.43182476876</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>The applications table scrolls sideways on my phone and the status column is off screen, so I cannot tell which ones are still pending without rotating.</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Linh Nguyễn</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr"/>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>/app/applications</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>390 x 664</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="n"/>
+      <c r="J11" s="4" t="inlineStr"/>
+      <c r="K11" s="4" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="n">
+        <v>46294.3901581021</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Praise</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>Signed up and posted my first bounty in under fifteen minutes with no support contact. The step that asks what you are here for made the rest of it make sense.</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Piotr Kaczmarek</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr"/>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>/app/onboarding</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>1728 x 962</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="n"/>
+      <c r="J12" s="4" t="inlineStr"/>
+      <c r="K12" s="4" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="n">
+        <v>46294.34849143543</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Handled</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>In the admin feedback queue, changing the status filter and then pressing back does not restore the previous filter, it leaves the admin section entirely.</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Priya Nair</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr"/>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>/admin/feedback</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>1920 x 947</t>
+        </is>
+      </c>
+      <c r="I13" s="5" t="n">
+        <v>46295.47349143543</v>
+      </c>
+      <c r="J13" s="4" t="inlineStr">
+        <is>
+          <t>Morgan Reyes</t>
+        </is>
+      </c>
+      <c r="K13" s="4" t="inlineStr">
+        <is>
+          <t>The filter is not in the URL. Agreed it should be — queued behind the reports queue work.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="n">
+        <v>46294.26927628784</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>It would help enormously to see the reward converted to a local currency estimate next to the XLM amount. I am doing the conversion in another tab every time.</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>Kwame Asante</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr"/>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>/bounties/build-a-bridge-between-a-mobile-money-api-and-on-ledger-settlement-9b98c0</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>360 x 720</t>
+        </is>
+      </c>
+      <c r="I14" s="4" t="n"/>
+      <c r="J14" s="4" t="inlineStr"/>
+      <c r="K14" s="4" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="n">
+        <v>46294.22349143543</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Praise</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Being able to read everything and apply without connecting a wallet first is a relief. Most sites like this put the wallet in front of the door.</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Anonymous</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>first.look.2026@example.test</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>412 x 823</t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="n"/>
+      <c r="J15" s="4" t="inlineStr"/>
+      <c r="K15" s="4" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="n">
+        <v>46294.18182476876</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Handled</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>My saved search says three new matches but opening it shows nothing new. I think the count is not being cleared when I view it from the sidebar rather than the saved page.</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>Ravi Deshmukh</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr"/>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>/app/saved</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>1366 x 625</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="n">
+        <v>46294.55682476876</v>
+      </c>
+      <c r="J16" s="4" t="inlineStr">
+        <is>
+          <t>Morgan Reyes</t>
+        </is>
+      </c>
+      <c r="K16" s="4" t="inlineStr">
+        <is>
+          <t>Reproduced. The sidebar link was not marking the search viewed. Fix is in review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="n">
+        <v>46294.1401581021</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Handled</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Question rather than feedback: if I complete a bounty, do you produce anything I can give my accountant, or do I invoice the requester myself?</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>Sofia Marchetti</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr"/>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>/app/payments</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>1920 x 947</t>
+        </is>
+      </c>
+      <c r="I17" s="5" t="n">
+        <v>46294.68182476876</v>
+      </c>
+      <c r="J17" s="4" t="inlineStr">
+        <is>
+          <t>Priya Nair</t>
+        </is>
+      </c>
+      <c r="K17" s="4" t="inlineStr">
+        <is>
+          <t>Answered by email: the requester pays directly on-chain, the platform is not a party, and the transaction record is exportable. Suggested we add this to the FAQ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="n">
+        <v>46294.10260962117</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Let me follow a bounty's questions without bookmarking it. I want the answers but I am not saving it to apply later.</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Maya Goldberg</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr"/>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>/bounties/build-a-visual-editor-for-multisig-signing-policies-9be393</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>1512 x 857</t>
+        </is>
+      </c>
+      <c r="I18" s="4" t="n"/>
+      <c r="J18" s="4" t="inlineStr"/>
+      <c r="K18" s="4" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="n">
+        <v>46294.05682476876</v>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>The analytics page takes about eleven seconds to load for me and shows an empty chart area the whole time, so it looks broken rather than slow.</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>Zanele Mthembu</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr"/>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>/app/analytics</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>1920 x 947</t>
+        </is>
+      </c>
+      <c r="I19" s="4" t="n"/>
+      <c r="J19" s="4" t="inlineStr"/>
+      <c r="K19" s="4" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="n">
+        <v>46294.0151581021</v>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Praise</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>The marketplace is fast on a bad connection, which is not something I get to say often. Filters apply without a full page reload and nothing jumps around while it loads.</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>Aminata Traoré</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr"/>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>/bounties</t>
+        </is>
+      </c>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>360 x 720</t>
+        </is>
+      </c>
+      <c r="I20" s="4" t="n"/>
+      <c r="J20" s="4" t="inlineStr"/>
+      <c r="K20" s="4" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="n">
+        <v>46293.9359429545</v>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Handled</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>The application deadline on a bounty shows a date with no timezone. I applied on what I thought was the last day and it had already closed. Please show the time and the zone.</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>Karan Mehta</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr"/>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>/bounties/security-review-of-a-soroban-token-vesting-contract-c15755</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>1512 x 857</t>
+        </is>
+      </c>
+      <c r="I21" s="5" t="n">
+        <v>46294.39427628784</v>
+      </c>
+      <c r="J21" s="4" t="inlineStr">
+        <is>
+          <t>Priya Nair</t>
+        </is>
+      </c>
+      <c r="K21" s="4" t="inlineStr">
+        <is>
+          <t>Real problem. Logged for the next UI pass; deadlines will render with the local time and an explicit UTC offset.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="n">
+        <v>46293.8901581021</v>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>When I have picked someone, let me decline the other applicants in one action with one shared message. Doing it one at a time makes me put it off, which is worse for them.</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>Aurora Ledger</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr"/>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>/app/bounties</t>
+        </is>
+      </c>
+      <c r="H22" s="4" t="inlineStr">
+        <is>
+          <t>1536 x 730</t>
+        </is>
+      </c>
+      <c r="I22" s="4" t="n"/>
+      <c r="J22" s="4" t="inlineStr"/>
+      <c r="K22" s="4" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="n">
+        <v>46293.84849143543</v>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Handled</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>There is a bounty in the design category that is clearly a development task. Not sure whether to report it or whether miscategorising is just something that happens.</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>Inès Moreau</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr"/>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>/bounties</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>1536 x 730</t>
+        </is>
+      </c>
+      <c r="I23" s="5" t="n">
+        <v>46294.1401581021</v>
+      </c>
+      <c r="J23" s="4" t="inlineStr">
+        <is>
+          <t>Priya Nair</t>
+        </is>
+      </c>
+      <c r="K23" s="4" t="inlineStr">
+        <is>
+          <t>Checked it, agreed, and asked the requester to recategorise rather than acting unilaterally. They did.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="n">
+        <v>46293.80682476876</v>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Handled</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>A saved cover letter template would save me ten minutes per application. Not a generic one — my own text that I edit each time.</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>Amara Diallo</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr"/>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>/app/applications</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t>1512 x 857</t>
+        </is>
+      </c>
+      <c r="I24" s="5" t="n">
+        <v>46294.68182476876</v>
+      </c>
+      <c r="J24" s="4" t="inlineStr">
+        <is>
+          <t>Priya Nair</t>
+        </is>
+      </c>
+      <c r="K24" s="4" t="inlineStr">
+        <is>
+          <t>Good idea and cheap. Added to the applications backlog with her wording attached.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="n">
+        <v>46293.76927628784</v>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>A code block in a question renders as a single long line on mobile instead of scrolling inside its own box. It pushes the whole page sideways.</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>Ahmed Farouk</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr"/>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>/bounties/build-a-resilient-orderbook-streaming-client-in-go-0a13dd</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>412 x 823</t>
+        </is>
+      </c>
+      <c r="I25" s="4" t="n"/>
+      <c r="J25" s="4" t="inlineStr"/>
+      <c r="K25" s="4" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="n">
+        <v>46293.72349143543</v>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Praise</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>Handled</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>The page explaining what happens to the money is unusually honest. It says what the platform cannot do, which is the part everyone else leaves out.</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>Mei-Lin Koh</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr"/>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>/how-it-works</t>
+        </is>
+      </c>
+      <c r="H26" s="4" t="inlineStr">
+        <is>
+          <t>1920 x 947</t>
+        </is>
+      </c>
+      <c r="I26" s="5" t="n">
+        <v>46294.1401581021</v>
+      </c>
+      <c r="J26" s="4" t="inlineStr">
+        <is>
+          <t>Morgan Reyes</t>
+        </is>
+      </c>
+      <c r="K26" s="4" t="inlineStr">
+        <is>
+          <t>Passed to the person who wrote it. Nothing to action, worth reading.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="n">
+        <v>46293.6401581021</v>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>Handled</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>A reward of 1234.5678901 shows as 1234.57 on the card and 1234.5678901 on the detail page. One of those is wrong and for money I would rather see the full value everywhere.</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>Felipe Cardozo</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr"/>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>/bounties</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="inlineStr">
+        <is>
+          <t>2560 x 1329</t>
+        </is>
+      </c>
+      <c r="I27" s="5" t="n">
+        <v>46294.22349143543</v>
+      </c>
+      <c r="J27" s="4" t="inlineStr">
+        <is>
+          <t>Priya Nair</t>
+        </is>
+      </c>
+      <c r="K27" s="4" t="inlineStr">
+        <is>
+          <t>Deliberate on the card for space, but he is right that it should be obvious it is truncated. Passed to design.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="n">
+        <v>46293.59849143543</v>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>Let me choose what time the daily digest arrives. Mine turns up at 2am and is buried by morning.</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>Dilnoza Usmanova</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr"/>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>/app/settings</t>
+        </is>
+      </c>
+      <c r="H28" s="4" t="inlineStr">
+        <is>
+          <t>360 x 720</t>
+        </is>
+      </c>
+      <c r="I28" s="4" t="n"/>
+      <c r="J28" s="4" t="inlineStr"/>
+      <c r="K28" s="4" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="n">
+        <v>46293.5151581021</v>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>Handled</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>Let contributors show a timezone on their profile. As a requester I care a lot whether someone overlaps with my working day and there is no way to tell.</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>Hiroshi Endō</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr"/>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>/u/kai-tanaka</t>
+        </is>
+      </c>
+      <c r="H29" s="4" t="inlineStr">
+        <is>
+          <t>1728 x 962</t>
+        </is>
+      </c>
+      <c r="I29" s="5" t="n">
+        <v>46294.7651581021</v>
+      </c>
+      <c r="J29" s="4" t="inlineStr">
+        <is>
+          <t>Morgan Reyes</t>
+        </is>
+      </c>
+      <c r="K29" s="4" t="inlineStr">
+        <is>
+          <t>Agreed, and it pairs well with the availability field already sketched. On the profile roadmap for next quarter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="n">
+        <v>46293.47349143543</v>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Praise</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>Handled</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>Reviewed six applications on my phone on a train and did not once wish I had a laptop. The review screens hold up at this size.</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>Théo Lambert</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr"/>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>/app/bounties</t>
+        </is>
+      </c>
+      <c r="H30" s="4" t="inlineStr">
+        <is>
+          <t>390 x 664</t>
+        </is>
+      </c>
+      <c r="I30" s="5" t="n">
+        <v>46294.30682476876</v>
+      </c>
+      <c r="J30" s="4" t="inlineStr">
+        <is>
+          <t>Morgan Reyes</t>
+        </is>
+      </c>
+      <c r="K30" s="4" t="inlineStr">
+        <is>
+          <t>Shared with the team that did the mobile pass. Closing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="n">
+        <v>46293.43182476876</v>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>A bounty with a very long title overflows its card on the marketplace grid and covers the reward amount underneath it.</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>Carmen Ortiz</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr"/>
+      <c r="G31" s="4" t="inlineStr">
+        <is>
+          <t>/bounties</t>
+        </is>
+      </c>
+      <c r="H31" s="4" t="inlineStr">
+        <is>
+          <t>1024 x 1292</t>
+        </is>
+      </c>
+      <c r="I31" s="4" t="n"/>
+      <c r="J31" s="4" t="inlineStr"/>
+      <c r="K31" s="4" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="n">
+        <v>46293.3901581021</v>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>Do you test with screen readers as part of your release process, or is accessibility handled by audits after the fact? Asking before I recommend this to a client.</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t>Zara Iqbal</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr"/>
+      <c r="G32" s="4" t="inlineStr">
+        <is>
+          <t>/about</t>
+        </is>
+      </c>
+      <c r="H32" s="4" t="inlineStr">
+        <is>
+          <t>1440 x 768</t>
+        </is>
+      </c>
+      <c r="I32" s="4" t="n"/>
+      <c r="J32" s="4" t="inlineStr"/>
+      <c r="K32" s="4" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="n">
+        <v>46293.30682476876</v>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>An RSS or Atom feed per saved search would let me read new bounties where I already read everything else, without another email subscription.</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>Tobias Berg</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr"/>
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t>/app/saved</t>
+        </is>
+      </c>
+      <c r="H33" s="4" t="inlineStr">
+        <is>
+          <t>2560 x 1329</t>
+        </is>
+      </c>
+      <c r="I33" s="4" t="n"/>
+      <c r="J33" s="4" t="inlineStr"/>
+      <c r="K33" s="4" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="n">
+        <v>46293.22349143543</v>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Praise</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>I navigated the whole application flow with a keyboard and a screen reader without getting stuck once. That is rare enough that I wanted to say so.</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>Aiko Matsumoto</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr"/>
+      <c r="G34" s="4" t="inlineStr">
+        <is>
+          <t>/app/applications</t>
+        </is>
+      </c>
+      <c r="H34" s="4" t="inlineStr">
+        <is>
+          <t>1440 x 768</t>
+        </is>
+      </c>
+      <c r="I34" s="4" t="n"/>
+      <c r="J34" s="4" t="inlineStr"/>
+      <c r="K34" s="4" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="n">
+        <v>46293.18182476876</v>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>Handled</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>The skills field on my profile has no autocomplete, so I typed react.js and the marketplace filter for react does not match me. Two spellings of the same skill should not split the list.</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>Anonymous</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>d.bakker.dev@example.test</t>
+        </is>
+      </c>
+      <c r="G35" s="4" t="inlineStr">
+        <is>
+          <t>/app/profile</t>
+        </is>
+      </c>
+      <c r="H35" s="4" t="inlineStr">
+        <is>
+          <t>1920 x 947</t>
+        </is>
+      </c>
+      <c r="I35" s="5" t="n">
+        <v>46293.97349143543</v>
+      </c>
+      <c r="J35" s="4" t="inlineStr">
+        <is>
+          <t>Priya Nair</t>
+        </is>
+      </c>
+      <c r="K35" s="4" t="inlineStr">
+        <is>
+          <t>Merged the duplicate spellings in the skill graph and opened a ticket for an autocomplete on the field. Wrote back to say so.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="n">
+        <v>46293.09849143543</v>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>Handled</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>A preview tab on the bounty description editor. I write Markdown fine but I would still like to see it before publishing to sixty people.</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>Anneke Visser</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="inlineStr"/>
+      <c r="G36" s="4" t="inlineStr">
+        <is>
+          <t>/app/bounties/create</t>
+        </is>
+      </c>
+      <c r="H36" s="4" t="inlineStr">
+        <is>
+          <t>1920 x 947</t>
+        </is>
+      </c>
+      <c r="I36" s="5" t="n">
+        <v>46293.7651581021</v>
+      </c>
+      <c r="J36" s="4" t="inlineStr">
+        <is>
+          <t>Priya Nair</t>
+        </is>
+      </c>
+      <c r="K36" s="4" t="inlineStr">
+        <is>
+          <t>Already half built behind a flag. Told her roughly when it lands.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="n">
+        <v>46293.05682476876</v>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>Handled</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>Is there any guidance on the tax treatment of a bounty reward in the EU? Not asking for advice, just whether anything exists that I could read.</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>Anonymous</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>questions.eu.2026@example.test</t>
+        </is>
+      </c>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>/guide</t>
+        </is>
+      </c>
+      <c r="H37" s="4" t="inlineStr">
+        <is>
+          <t>1366 x 625</t>
+        </is>
+      </c>
+      <c r="I37" s="5" t="n">
+        <v>46293.7651581021</v>
+      </c>
+      <c r="J37" s="4" t="inlineStr">
+        <is>
+          <t>Morgan Reyes</t>
+        </is>
+      </c>
+      <c r="K37" s="4" t="inlineStr">
+        <is>
+          <t>Replied that we do not publish tax guidance and cannot advise. Pointed at the transaction export as the record their accountant will want.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="n">
+        <v>46293.01927628784</v>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>Handled</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>In dark mode the secondary text on the bounty detail page fails contrast against the background. Measured it at about 3.1:1 where it needs 4.5:1.</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>Zara Iqbal</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="inlineStr"/>
+      <c r="G38" s="4" t="inlineStr">
+        <is>
+          <t>/bounties/wcag-2-2-aa-audit-of-three-funded-open-source-web-apps-6339a1</t>
+        </is>
+      </c>
+      <c r="H38" s="4" t="inlineStr">
+        <is>
+          <t>1728 x 962</t>
+        </is>
+      </c>
+      <c r="I38" s="5" t="n">
+        <v>46293.35260962117</v>
+      </c>
+      <c r="J38" s="4" t="inlineStr">
+        <is>
+          <t>Morgan Reyes</t>
+        </is>
+      </c>
+      <c r="K38" s="4" t="inlineStr">
+        <is>
+          <t>Confirmed with the same measurement. Token adjusted and the whole dark palette rechecked while we were in there.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="n">
+        <v>46292.93182476876</v>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>Handled</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>Is there a public API for the marketplace listings? I would like to mirror open bounties into our internal board rather than asking people to check two places.</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>Nova Labs</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr"/>
+      <c r="G39" s="4" t="inlineStr">
+        <is>
+          <t>/guide</t>
+        </is>
+      </c>
+      <c r="H39" s="4" t="inlineStr">
+        <is>
+          <t>1728 x 962</t>
+        </is>
+      </c>
+      <c r="I39" s="5" t="n">
+        <v>46293.3901581021</v>
+      </c>
+      <c r="J39" s="4" t="inlineStr">
+        <is>
+          <t>Morgan Reyes</t>
+        </is>
+      </c>
+      <c r="K39" s="4" t="inlineStr">
+        <is>
+          <t>Pointed at the public listing endpoints and the rate limits. Asked them to tell us if the limits are too tight for a mirror.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="n">
+        <v>46292.8901581021</v>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>Handled</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>I spent forty minutes writing a bounty description, the session expired while I was reading something else, and hitting save took me to the login page and threw the whole thing away.</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>Lucas Ferreira</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="inlineStr"/>
+      <c r="G40" s="4" t="inlineStr">
+        <is>
+          <t>/app/bounties/create</t>
+        </is>
+      </c>
+      <c r="H40" s="4" t="inlineStr">
+        <is>
+          <t>1728 x 962</t>
+        </is>
+      </c>
+      <c r="I40" s="5" t="n">
+        <v>46293.18182476876</v>
+      </c>
+      <c r="J40" s="4" t="inlineStr">
+        <is>
+          <t>Morgan Reyes</t>
+        </is>
+      </c>
+      <c r="K40" s="4" t="inlineStr">
+        <is>
+          <t>Worst kind of bug. The create form now keeps a local draft and restores it after sign-in. Apologised and asked him to try again.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="n">
+        <v>46292.84849143543</v>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>Praise</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>Handled</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>Whoever wrote the empty state on the saved page — thank you. It told me what to do next instead of just telling me the list was empty.</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>Daniela Vargas</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr"/>
+      <c r="G41" s="4" t="inlineStr">
+        <is>
+          <t>/app/saved</t>
+        </is>
+      </c>
+      <c r="H41" s="4" t="inlineStr">
+        <is>
+          <t>390 x 664</t>
+        </is>
+      </c>
+      <c r="I41" s="5" t="n">
+        <v>46293.59849143543</v>
+      </c>
+      <c r="J41" s="4" t="inlineStr">
+        <is>
+          <t>Priya Nair</t>
+        </is>
+      </c>
+      <c r="K41" s="4" t="inlineStr">
+        <is>
+          <t>Forwarded to content design. No action needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="n">
+        <v>46292.72349143543</v>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>Handled</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>I got the same application-received notification twice, about four seconds apart, for one application.</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="inlineStr">
+        <is>
+          <t>Arun Ramaswamy</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="inlineStr"/>
+      <c r="G42" s="4" t="inlineStr">
+        <is>
+          <t>/app/notifications</t>
+        </is>
+      </c>
+      <c r="H42" s="4" t="inlineStr">
+        <is>
+          <t>1536 x 730</t>
+        </is>
+      </c>
+      <c r="I42" s="5" t="n">
+        <v>46292.97349143543</v>
+      </c>
+      <c r="J42" s="4" t="inlineStr">
+        <is>
+          <t>Morgan Reyes</t>
+        </is>
+      </c>
+      <c r="K42" s="4" t="inlineStr">
+        <is>
+          <t>Traced to a redelivered event with a null source id, which skipped the uniqueness check. Fixed at the consumer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="n">
+        <v>46292.68182476876</v>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>Handled</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>I want to close my account but I have one open application. Does closing withdraw it, and does the requester see that I left?</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>Pablo Navarro</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="inlineStr"/>
+      <c r="G43" s="4" t="inlineStr">
+        <is>
+          <t>/app/privacy</t>
+        </is>
+      </c>
+      <c r="H43" s="4" t="inlineStr">
+        <is>
+          <t>1512 x 857</t>
+        </is>
+      </c>
+      <c r="I43" s="5" t="n">
+        <v>46293.05682476876</v>
+      </c>
+      <c r="J43" s="4" t="inlineStr">
+        <is>
+          <t>Priya Nair</t>
+        </is>
+      </c>
+      <c r="K43" s="4" t="inlineStr">
+        <is>
+          <t>Explained the deletion flow: open applications are withdrawn and the requester sees a withdrawal, not a name. He decided to keep the account for now.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="n">
+        <v>46292.59849143543</v>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>I would like to withdraw an application with a short note to the requester rather than silently. It feels rude to just disappear when my availability changes.</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr">
+        <is>
+          <t>Hana Suzuki</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="inlineStr"/>
+      <c r="G44" s="4" t="inlineStr">
+        <is>
+          <t>/app/applications</t>
+        </is>
+      </c>
+      <c r="H44" s="4" t="inlineStr">
+        <is>
+          <t>412 x 823</t>
+        </is>
+      </c>
+      <c r="I44" s="4" t="n"/>
+      <c r="J44" s="4" t="inlineStr"/>
+      <c r="K44" s="4" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="n">
+        <v>46292.5151581021</v>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Praise</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>The audit log actually records who did what and when, in a format I can read. I have used admin tools where that was a wishlist item.</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="inlineStr">
+        <is>
+          <t>Priya Nair</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="inlineStr"/>
+      <c r="G45" s="4" t="inlineStr">
+        <is>
+          <t>/admin/audit-logs</t>
+        </is>
+      </c>
+      <c r="H45" s="4" t="inlineStr">
+        <is>
+          <t>1920 x 947</t>
+        </is>
+      </c>
+      <c r="I45" s="4" t="n"/>
+      <c r="J45" s="4" t="inlineStr"/>
+      <c r="K45" s="4" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="n">
+        <v>46292.43182476876</v>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>Handled</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>Clicking the verification link in my email logs me out and sends me to sign in, and after signing in the banner still says my address is unverified. Took me three tries to get through.</t>
+        </is>
+      </c>
+      <c r="E46" s="4" t="inlineStr">
+        <is>
+          <t>Anonymous</t>
+        </is>
+      </c>
+      <c r="F46" s="4" t="inlineStr">
+        <is>
+          <t>tanvir.h.mail@example.test</t>
+        </is>
+      </c>
+      <c r="G46" s="4" t="inlineStr">
+        <is>
+          <t>/verify-email</t>
+        </is>
+      </c>
+      <c r="H46" s="4" t="inlineStr">
+        <is>
+          <t>390 x 664</t>
+        </is>
+      </c>
+      <c r="I46" s="5" t="n">
+        <v>46292.6401581021</v>
+      </c>
+      <c r="J46" s="4" t="inlineStr">
+        <is>
+          <t>Morgan Reyes</t>
+        </is>
+      </c>
+      <c r="K46" s="4" t="inlineStr">
+        <is>
+          <t>Caused by the token being consumed before the session was established on mobile Safari. Fixed and verified on a real device.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="n">
+        <v>46292.34849143543</v>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>I appear to have signed up twice with two addresses and I cannot merge them. The one with my applications is the one I want to keep.</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="inlineStr">
+        <is>
+          <t>Anonymous</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>m.lindgren.two@example.test</t>
+        </is>
+      </c>
+      <c r="G47" s="4" t="inlineStr">
+        <is>
+          <t>/app/settings</t>
+        </is>
+      </c>
+      <c r="H47" s="4" t="inlineStr">
+        <is>
+          <t>412 x 823</t>
+        </is>
+      </c>
+      <c r="I47" s="4" t="n"/>
+      <c r="J47" s="4" t="inlineStr"/>
+      <c r="K47" s="4" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="n">
+        <v>46292.26927628784</v>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>Handled</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>A print stylesheet for a bounty page. Two of my colleagues review these on paper and the current print output includes the whole navigation.</t>
+        </is>
+      </c>
+      <c r="E48" s="4" t="inlineStr">
+        <is>
+          <t>Anonymous</t>
+        </is>
+      </c>
+      <c r="F48" s="4" t="inlineStr">
+        <is>
+          <t>ops.review.desk@example.test</t>
+        </is>
+      </c>
+      <c r="G48" s="4" t="inlineStr">
+        <is>
+          <t>/bounties/redesign-the-daily-settlement-report-for-the-operations-desk-6726ab</t>
+        </is>
+      </c>
+      <c r="H48" s="4" t="inlineStr">
+        <is>
+          <t>1440 x 768</t>
+        </is>
+      </c>
+      <c r="I48" s="5" t="n">
+        <v>46293.3109429545</v>
+      </c>
+      <c r="J48" s="4" t="inlineStr">
+        <is>
+          <t>Priya Nair</t>
+        </is>
+      </c>
+      <c r="K48" s="4" t="inlineStr">
+        <is>
+          <t>Small and worth doing. Added to the design-polish list.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="n">
+        <v>46292.18182476876</v>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>Praise</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="D49" s="4" t="inlineStr">
+        <is>
+          <t>The privacy page tells me exactly what is stored and lets me export it without emailing anyone. Genuinely the first time I have seen that work in one click.</t>
+        </is>
+      </c>
+      <c r="E49" s="4" t="inlineStr">
+        <is>
+          <t>Nina Schneider</t>
+        </is>
+      </c>
+      <c r="F49" s="4" t="inlineStr"/>
+      <c r="G49" s="4" t="inlineStr">
+        <is>
+          <t>/app/privacy</t>
+        </is>
+      </c>
+      <c r="H49" s="4" t="inlineStr">
+        <is>
+          <t>2560 x 1329</t>
+        </is>
+      </c>
+      <c r="I49" s="4" t="n"/>
+      <c r="J49" s="4" t="inlineStr"/>
+      <c r="K49" s="4" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="n">
+        <v>46292.09849143543</v>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t>Handled</t>
+        </is>
+      </c>
+      <c r="D50" s="4" t="inlineStr">
+        <is>
+          <t>Some signal of who has actually completed work would help me decide between five similar applications. Not a score, just something verifiable.</t>
+        </is>
+      </c>
+      <c r="E50" s="4" t="inlineStr">
+        <is>
+          <t>Helio Collective</t>
+        </is>
+      </c>
+      <c r="F50" s="4" t="inlineStr"/>
+      <c r="G50" s="4" t="inlineStr">
+        <is>
+          <t>/app/bounties</t>
+        </is>
+      </c>
+      <c r="H50" s="4" t="inlineStr">
+        <is>
+          <t>1728 x 962</t>
+        </is>
+      </c>
+      <c r="I50" s="5" t="n">
+        <v>46292.59849143543</v>
+      </c>
+      <c r="J50" s="4" t="inlineStr">
+        <is>
+          <t>Morgan Reyes</t>
+        </is>
+      </c>
+      <c r="K50" s="4" t="inlineStr">
+        <is>
+          <t>This is what the attestation work is for. Explained the plan and pointed at the public attestation page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="n">
+        <v>46292.0151581021</v>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>Handled</t>
+        </is>
+      </c>
+      <c r="D51" s="4" t="inlineStr">
+        <is>
+          <t>We run a developer community of about 4,000 people in South East Asia and would like to talk about putting bounties in front of them. Who should I write to?</t>
+        </is>
+      </c>
+      <c r="E51" s="4" t="inlineStr">
+        <is>
+          <t>Anonymous</t>
+        </is>
+      </c>
+      <c r="F51" s="4" t="inlineStr">
+        <is>
+          <t>programs.sea.network@example.test</t>
+        </is>
+      </c>
+      <c r="G51" s="4" t="inlineStr">
+        <is>
+          <t>/about</t>
+        </is>
+      </c>
+      <c r="H51" s="4" t="inlineStr">
+        <is>
+          <t>1920 x 947</t>
+        </is>
+      </c>
+      <c r="I51" s="5" t="n">
+        <v>46292.97349143543</v>
+      </c>
+      <c r="J51" s="4" t="inlineStr">
+        <is>
+          <t>Morgan Reyes</t>
+        </is>
+      </c>
+      <c r="K51" s="4" t="inlineStr">
+        <is>
+          <t>Not a support request. Forwarded to partnerships and replied with an introduction.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K2"/>
+  <autoFilter ref="A1:K51"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1110,7 +5415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1121,6 +5426,9 @@
     <col width="22" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1138,45 +5446,60 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>Name</t>
+          <t>Full name</t>
         </is>
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Email address</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>Stellar wallet address</t>
+          <t>Stellar wallet address (public key)</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>How would you rate BountyFlow?</t>
+          <t>How did you use BountyFlow?</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>What worked well?</t>
+          <t>Overall rating</t>
         </is>
       </c>
       <c r="G3" s="1" t="inlineStr">
         <is>
-          <t>What got in your way?</t>
+          <t>Ease of connecting a wallet and moving money</t>
         </is>
       </c>
       <c r="H3" s="1" t="inlineStr">
         <is>
-          <t>What should we build next?</t>
+          <t>Likelihood to recommend</t>
+        </is>
+      </c>
+      <c r="I3" s="1" t="inlineStr">
+        <is>
+          <t>Kind of feedback</t>
+        </is>
+      </c>
+      <c r="J3" s="1" t="inlineStr">
+        <is>
+          <t>What worked, and what did not?</t>
+        </is>
+      </c>
+      <c r="K3" s="1" t="inlineStr">
+        <is>
+          <t>If you could change one thing, what would it be?</t>
         </is>
       </c>
     </row>
     <row r="4"/>
   </sheetData>
-  <autoFilter ref="A3:H3"/>
+  <autoFilter ref="A3:K3"/>
   <mergeCells count="1">
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A1:K1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>